<commit_message>
feat(social-intelligence): add AI Vision Poster OCR, Registration Form Status Inspector, 52-page Campus Watchlist Poller & auto-upload GitHub secret
</commit_message>
<xml_diff>
--- a/data/aiesec_egypt_events_latest.xlsx
+++ b/data/aiesec_egypt_events_latest.xlsx
@@ -1517,7 +1517,9 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>Come join us in Urban court for a chill boardgame night, where we have fun and make new friends. Zero experience in games needed, as I will be your host and game master introducing you to games. Join our WhatsApp group
+          <t>Come join us in Urban court for a chill boardgame night, where we have fun and make new friends.
+Zero experience in games needed, as I will be your host and game master introducing you to games.
+Join our WhatsApp group
 [https://chat.whatsapp.com/CrOryPPzVTC0j2NLNq75Gj](https://chat.whatsapp.com/Cr</t>
         </is>
       </c>
@@ -1611,11 +1613,14 @@
       <c r="R13" t="inlineStr">
         <is>
           <t>Book Your Spot:
-https://www.instagram.com/TalentRiseAcademy/ You came to meet new people... and somehow ended up oversharing over a card game 💛🃏 This time, we’re keeping it light:
+https://www.instagram.com/TalentRiseAcademy/
+You came to meet new people... and somehow ended up oversharing over a card game 💛🃏
+This time, we’re keeping it light:
 ✨ABtalks Card Games
 😂 Laughs &amp; good vibes
 🫱🏻‍🫲🏼New people
-💬Conversations that actually go somewhere No pressure. No a</t>
+💬Conversations that actually go somewhere
+No pressure. No a</t>
         </is>
       </c>
     </row>
@@ -1707,7 +1712,8 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>We all have a handful of automatic moves we make in close relationships. They fire faster than thought. They feel like personality rather than choice. From the inside, you cannot see your own strategy.
+          <t>We all have a handful of automatic moves we make in close relationships. They fire faster than thought. They feel like personality rather than choice.
+From the inside, you cannot see your own strategy.
 In this session I will walk you through all eight, one by one. Most people recognise themselves i</t>
         </is>
       </c>
@@ -1800,7 +1806,11 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>## What you'll learn * Build Advanced Workflows Without Coding Use MCP connectors and plugins to link Claude to your daily apps and automate tasks without writing code. * Master Multi-Agent Systems Learn simple frameworks to coordinate multiple AI assistants for handling complex, multi-step proj</t>
+          <t>## What you'll learn
+* Build Advanced Workflows Without Coding
+Use MCP connectors and plugins to link Claude to your daily apps and automate tasks without writing code.
+* Master Multi-Agent Systems
+Learn simple frameworks to coordinate multiple AI assistants for handling complex, multi-step proj</t>
         </is>
       </c>
     </row>
@@ -2075,12 +2085,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ragheb Allama</t>
+          <t>Omar kint X Room Garden City</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Oct 08 · 05:30 PM</t>
+          <t>Thu, 08 Oct, 2026 - 08:00 PM</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2090,12 +2100,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Porto Elsokhna</t>
+          <t>ROOM Art Space &amp; Cafe</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>TicketsMarche</t>
+          <t>AllEvents</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2110,7 +2120,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>3000.00 EGP</t>
+          <t>Registration / Tickets</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2140,17 +2150,17 @@
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Amer Group</t>
+          <t>AllEvents Organizer</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>https://www.ticketsmarche.com/event/Ragheb_Allama_9438</t>
+          <t>https://allevents.in/cairo/omar-kint-x-room-garden-city/200030697848829</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>https://www.ticketsmarche.com/event/Ragheb_Allama_9438</t>
+          <t>https://allevents.in/cairo/omar-kint-x-room-garden-city/200030697848829</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
@@ -2158,21 +2168,17 @@
           <t>100% Verified Real</t>
         </is>
       </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>Ragheb Allama organized by Amer Group. Tickets available on TicketsMarche (3000.00 EGP). Venue: Porto Elsokhna.</t>
-        </is>
-      </c>
+      <c r="R19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Exclusive Material Tryout by Mohamed Helmy</t>
+          <t>Ragheb Allama</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Oct 08 · 08:30 PM</t>
+          <t>Oct 08 · 05:30 PM</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2182,7 +2188,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Teatro 90</t>
+          <t>Porto Elsokhna</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2202,7 +2208,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>999.00 EGP</t>
+          <t>3000.00 EGP</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2232,17 +2238,17 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Helmy manX teatro 90</t>
+          <t>Amer Group</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>https://www.ticketsmarche.com/event/exclusive-material-tryout-by-mohamed-helmy_9501</t>
+          <t>https://www.ticketsmarche.com/event/Ragheb_Allama_9438</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>https://www.ticketsmarche.com/event/exclusive-material-tryout-by-mohamed-helmy_9501</t>
+          <t>https://www.ticketsmarche.com/event/Ragheb_Allama_9438</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
@@ -2252,14 +2258,14 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>Exclusive Material Tryout by Mohamed Helmy organized by Helmy manX teatro 90. Tickets available on TicketsMarche (999.00 EGP). Venue: Teatro 90.</t>
+          <t>Ragheb Allama organized by Amer Group. Tickets available on TicketsMarche (3000.00 EGP). Venue: Porto Elsokhna.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Al-Dahdira Play</t>
+          <t>Exclusive Material Tryout by Mohamed Helmy</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2274,7 +2280,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>El Rihany Theater</t>
+          <t>Teatro 90</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2294,7 +2300,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>100.00 EGP</t>
+          <t>999.00 EGP</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -2324,17 +2330,17 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>sokseh</t>
+          <t>Helmy manX teatro 90</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>https://www.ticketsmarche.com/event/Al-Dahdira_9536</t>
+          <t>https://www.ticketsmarche.com/event/exclusive-material-tryout-by-mohamed-helmy_9501</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>https://www.ticketsmarche.com/event/Al-Dahdira_9536</t>
+          <t>https://www.ticketsmarche.com/event/exclusive-material-tryout-by-mohamed-helmy_9501</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
@@ -2344,19 +2350,19 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Al-Dahdira Play organized by sokseh. Tickets available on TicketsMarche (100.00 EGP). Venue: El Rihany Theater.</t>
+          <t>Exclusive Material Tryout by Mohamed Helmy organized by Helmy manX teatro 90. Tickets available on TicketsMarche (999.00 EGP). Venue: Teatro 90.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Omar kint X Room Garden City</t>
+          <t>Al-Dahdira Play</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Thu, 08 Oct, 2026 - 08:00 PM</t>
+          <t>Oct 08 · 08:30 PM</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2366,12 +2372,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>ROOM Art Space &amp; Cafe</t>
+          <t>El Rihany Theater</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>AllEvents</t>
+          <t>TicketsMarche</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -2386,7 +2392,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Registration / Tickets</t>
+          <t>100.00 EGP</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2416,17 +2422,17 @@
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>AllEvents Organizer</t>
+          <t>sokseh</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>https://allevents.in/cairo/omar-kint-x-room-garden-city/200030697848829</t>
+          <t>https://www.ticketsmarche.com/event/Al-Dahdira_9536</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>https://allevents.in/cairo/omar-kint-x-room-garden-city/200030697848829</t>
+          <t>https://www.ticketsmarche.com/event/Al-Dahdira_9536</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
@@ -2434,7 +2440,11 @@
           <t>100% Verified Real</t>
         </is>
       </c>
-      <c r="R22" t="inlineStr"/>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>Al-Dahdira Play organized by sokseh. Tickets available on TicketsMarche (100.00 EGP). Venue: El Rihany Theater.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2797,7 +2807,8 @@
       <c r="R26" t="inlineStr">
         <is>
           <t>A casual weekend meetup for good coffee, breakfast, and great conversations! ☕️🥐
-Every weekend, we’ll meet at Qahwa 5A, New Cairo to enjoy a relaxed morning, have some coffee and breakfast, and meet new people. No special requirements—just come with a good mood, an open mind, and a willingness to m</t>
+Every weekend, we’ll meet at Qahwa 5A, New Cairo to enjoy a relaxed morning, have some coffee and breakfast, and meet new people.
+No special requirements—just come with a good mood, an open mind, and a willingness to m</t>
         </is>
       </c>
     </row>
@@ -3068,27 +3079,27 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Leila Assal</t>
+          <t>Marioneta Show Season 29</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>8 and 9 Oct · 8:00 PM</t>
+          <t>Fri, 09 Oct, 2026 - 06:00 PM</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Giza</t>
+          <t>Cairo</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Cairo Cultural Hub</t>
+          <t>Galal El Sharkawy Theatre   مسرح جلال الشرقاوي</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>TicketsMarche</t>
+          <t>AllEvents</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -3103,7 +3114,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Free / Paid Tickets</t>
+          <t>Registration / Tickets</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -3133,17 +3144,17 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>film square</t>
+          <t>AllEvents Organizer</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>https://www.ticketsmarche.com/event/leila_assall</t>
+          <t>https://allevents.in/cairo/marioneta-show-season-29/200030776555736</t>
         </is>
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>https://www.ticketsmarche.com/event/leila_assall</t>
+          <t>https://allevents.in/cairo/marioneta-show-season-29/200030776555736</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -3151,36 +3162,32 @@
           <t>100% Verified Real</t>
         </is>
       </c>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>Leila Assal organized by film square. Tickets available on TicketsMarche (Free / Paid Tickets). Venue: Cairo Cultural Hub.</t>
-        </is>
-      </c>
+      <c r="R30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Marioneta Show Season 29</t>
+          <t>Leila Assal</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Fri, 09 Oct, 2026 - 06:00 PM</t>
+          <t>8 and 9 Oct · 8:00 PM</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Cairo</t>
+          <t>Giza</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Galal El Sharkawy Theatre   مسرح جلال الشرقاوي</t>
+          <t>Cairo Cultural Hub</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>AllEvents</t>
+          <t>TicketsMarche</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3195,7 +3202,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Registration / Tickets</t>
+          <t>Free / Paid Tickets</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -3225,17 +3232,17 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>AllEvents Organizer</t>
+          <t>film square</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>https://allevents.in/cairo/marioneta-show-season-29/200030776555736</t>
+          <t>https://www.ticketsmarche.com/event/leila_assall</t>
         </is>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>https://allevents.in/cairo/marioneta-show-season-29/200030776555736</t>
+          <t>https://www.ticketsmarche.com/event/leila_assall</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -3243,7 +3250,11 @@
           <t>100% Verified Real</t>
         </is>
       </c>
-      <c r="R31" t="inlineStr"/>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Leila Assal organized by film square. Tickets available on TicketsMarche (Free / Paid Tickets). Venue: Cairo Cultural Hub.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3529,12 +3540,12 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Sat, 10 Oct • 09:00 AM</t>
+          <t>Sat, 10 Oct, 2026 - 09:00 AM</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Tanta</t>
+          <t>Cairo</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -3574,7 +3585,7 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>⚠️ Clash</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
@@ -4777,8 +4788,10 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>Do you want to kick your public speaking skills up a couple of notches?
-Join Maadi Toastmasters Club and practice public speaking with professional speakers from all over the world to ace your next presentation. What's Maadi Toastmasters Club? A Toastmasters Club meeting is a learn-by-doing event</t>
+          <t xml:space="preserve">Do you want to kick your public speaking skills up a couple of notches?
+Join Maadi Toastmasters Club and practice public speaking with professional speakers from all over the world to ace your next presentation.
+What's Maadi Toastmasters Club?
+A Toastmasters Club meeting is a learn-by-doing event </t>
         </is>
       </c>
     </row>
@@ -4962,10 +4975,10 @@
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>Follow this link to join Caribou Coffee Meetup WhatsApp group: [https://chat.whatsapp.com/IZh4XcCOk1V2sXmIBqjYpq?s=sh&amp;p=a&amp;mlu=4](https://chat.whatsapp.com/IZh4XcCOk1V2sXmIBqjYpq?s=sh&amp;p=a&amp;mlu=4)
+          <t xml:space="preserve">Follow this link to join Caribou Coffee Meetup WhatsApp group: [https://chat.whatsapp.com/IZh4XcCOk1V2sXmIBqjYpq?s=sh&amp;p=a&amp;mlu=4](https://chat.whatsapp.com/IZh4XcCOk1V2sXmIBqjYpq?s=sh&amp;p=a&amp;mlu=4)
 For Inquiries WhatsApp ±2 01098292380
 When &amp; Where We Meet
-​Location: Caribou Coffee, East Walk Mall (New</t>
+​Location: Caribou Coffee, East Walk Mall (New </t>
         </is>
       </c>
     </row>
@@ -5423,7 +5436,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Heart Is Life Annual International Congress AIC 2026</t>
+          <t>Heart Is Life  Annual International Congress  AIC 2026</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -5596,7 +5609,9 @@
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>You write a spec, hand it to AI, and it gives you back a PR that looks right. But the implementation can be wrong! In the current tools (Kiro, spec-kit, Tessl), the spec is a Markdown file AI is supposed to follow. But AI can ignore the spec or misread it. So you end up testing everything by hand,</t>
+          <t>You write a spec, hand it to AI, and it gives you back a PR that looks right. But the implementation can be wrong!
+In the current tools (Kiro, spec-kit, Tessl), the spec is a Markdown file AI is supposed to follow. But AI can ignore the spec or misread it.
+So you end up testing everything by hand,</t>
         </is>
       </c>
     </row>
@@ -5689,7 +5704,8 @@
       <c r="R58" t="inlineStr">
         <is>
           <t>***Founders for Founders* brings you Real conversations for Entrepreneurs building Startups around the world. Every Wednesday.**
-*Talk it out, build it better.* * This is a special FREE weekly event for founders around the world: you can check out [The Founders for Founders Website](https://f4f.vc/</t>
+*Talk it out, build it better.*
+* This is a special FREE weekly event for founders around the world: you can check out [The Founders for Founders Website](https://f4f.vc/</t>
         </is>
       </c>
     </row>
@@ -6052,22 +6068,22 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>18th Annual Dialysis Conference The Cardiometabolic Summit</t>
+          <t>7th Annual Conference of Pharmacy</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct • 08:00 AM</t>
+          <t>Thu, 15 Oct, 2026 - 08:00 AM</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Tanta</t>
+          <t>Mansoura</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Novotel Cairo Airport (Po Box 8 Cairo Airport, Cairo, Cairo Governorate, Egypt)</t>
+          <t>Gzert El Ward Club</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -6122,12 +6138,12 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>https://allevents.in/heliopolis/18th-annual-dialysis-conference-the-cardiometabolic-summit/200030603841151</t>
+          <t>https://allevents.in/al-mansurah/7th-annual-conference-of-pharmacy/200030469186724</t>
         </is>
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>https://allevents.in/heliopolis/18th-annual-dialysis-conference-the-cardiometabolic-summit/200030603841151</t>
+          <t>https://allevents.in/al-mansurah/7th-annual-conference-of-pharmacy/200030469186724</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr">
@@ -6140,22 +6156,22 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>7th Annual Conference of Pharmacy</t>
+          <t>18th Annual Dialysis Conference The Cardiometabolic Summit</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct, 2026 - 08:00 AM</t>
+          <t>Thu, 15 Oct • 08:00 AM</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Mansoura</t>
+          <t>Tanta</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Gzert El Ward Club</t>
+          <t>Novotel Cairo Airport (Po Box 8 Cairo Airport, Cairo, Cairo Governorate, Egypt)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -6210,12 +6226,12 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>https://allevents.in/al-mansurah/7th-annual-conference-of-pharmacy/200030469186724</t>
+          <t>https://allevents.in/heliopolis/18th-annual-dialysis-conference-the-cardiometabolic-summit/200030603841151</t>
         </is>
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>https://allevents.in/al-mansurah/7th-annual-conference-of-pharmacy/200030469186724</t>
+          <t>https://allevents.in/heliopolis/18th-annual-dialysis-conference-the-cardiometabolic-summit/200030603841151</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr">
@@ -6590,12 +6606,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>I Want A Pet Dinosaur X Teatro 90</t>
+          <t>بيت السناري</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Oct 15 ,16</t>
+          <t>Thu, 15 Oct, 2026 - 08:00 PM</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -6605,12 +6621,12 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Teatro 90</t>
+          <t>Cairo, Egypt</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>TicketsMarche</t>
+          <t>AllEvents</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -6625,7 +6641,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Free / Paid Tickets</t>
+          <t>Registration / Tickets</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -6655,17 +6671,17 @@
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>Teatro 90 multiday</t>
+          <t>AllEvents Organizer</t>
         </is>
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>https://www.ticketsmarche.com/event/i_want-dinosaur_9488</t>
+          <t>https://allevents.in/cairo/حفل-مجاني-ميكروفون-21/200030783625739</t>
         </is>
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>https://www.ticketsmarche.com/event/i_want-dinosaur_9488</t>
+          <t>https://allevents.in/cairo/حفل-مجاني-ميكروفون-21/200030783625739</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr">
@@ -6673,21 +6689,17 @@
           <t>100% Verified Real</t>
         </is>
       </c>
-      <c r="R69" t="inlineStr">
-        <is>
-          <t>I Want A Pet Dinosaur X Teatro 90 organized by Teatro 90 multiday. Tickets available on TicketsMarche (Free / Paid Tickets). Venue: Teatro 90.</t>
-        </is>
-      </c>
+      <c r="R69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>بيت السناري</t>
+          <t>I Want A Pet Dinosaur X Teatro 90</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Thu, 15 Oct, 2026 - 08:00 PM</t>
+          <t>Oct 15 ,16</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -6697,12 +6709,12 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Cairo, Egypt</t>
+          <t>Teatro 90</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>AllEvents</t>
+          <t>TicketsMarche</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
@@ -6717,7 +6729,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Registration / Tickets</t>
+          <t>Free / Paid Tickets</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -6747,17 +6759,17 @@
       </c>
       <c r="N70" t="inlineStr">
         <is>
-          <t>AllEvents Organizer</t>
+          <t>Teatro 90 multiday</t>
         </is>
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>https://allevents.in/cairo/حفل-مجاني-ميكروفون-21/200030783625739</t>
+          <t>https://www.ticketsmarche.com/event/i_want-dinosaur_9488</t>
         </is>
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>https://allevents.in/cairo/حفل-مجاني-ميكروفون-21/200030783625739</t>
+          <t>https://www.ticketsmarche.com/event/i_want-dinosaur_9488</t>
         </is>
       </c>
       <c r="Q70" t="inlineStr">
@@ -6765,7 +6777,11 @@
           <t>100% Verified Real</t>
         </is>
       </c>
-      <c r="R70" t="inlineStr"/>
+      <c r="R70" t="inlineStr">
+        <is>
+          <t>I Want A Pet Dinosaur X Teatro 90 organized by Teatro 90 multiday. Tickets available on TicketsMarche (Free / Paid Tickets). Venue: Teatro 90.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -7314,12 +7330,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Chromatic Healing level 2</t>
+          <t>Cairo International Youth Language &amp; Cultural Exchange Night</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct • 05:00 PM</t>
+          <t>Oct 16, 2026 · 07:30 PM</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -7329,17 +7345,17 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Blue Lotus Wellbeing</t>
+          <t>Zamalek Youth Cultural Lounge, 26th of July Corridor, Zamalek, Cairo</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>AllEvents</t>
+          <t>Facebook Events</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>General Event</t>
+          <t>Campus &amp; Student Activities</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -7349,17 +7365,17 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Registration / Tickets</t>
+          <t>Free Admission / Open to All Youth</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>7.8</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>LOW</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -7369,27 +7385,27 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>campus, students, youth, education</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>General Monitoring for potential youth presence</t>
+          <t>Campus Outreach: Engage Student Attendees &amp; Student Union Partners</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>AllEvents Organizer</t>
+          <t>Make Friends Cairo Youth Community (@cairomakefriends)</t>
         </is>
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>https://allevents.in/heliopolis/chromatic-healing-level-2/200030583735256</t>
+          <t>https://www.facebook.com/groups/cairomakefriends</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>https://allevents.in/heliopolis/chromatic-healing-level-2/200030583735256</t>
+          <t>https://www.facebook.com/groups/cairomakefriends</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -7397,17 +7413,21 @@
           <t>100% Verified Real</t>
         </is>
       </c>
-      <c r="R77" t="inlineStr"/>
+      <c r="R77" t="inlineStr">
+        <is>
+          <t>The most active youth and international student cultural exchange gathering in Greater Cairo. Convenes university students, foreign exchange delegates, language learners, and young professionals for cross-cultural dialogues and networking in Zamalek.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Cairo International Youth Language &amp; Cultural Exchange Night</t>
+          <t>Chromatic Healing level 2</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Oct 16, 2026 · 07:30 PM</t>
+          <t>Fri, 16 Oct • 05:00 PM</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -7417,17 +7437,17 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Zamalek Youth Cultural Lounge, 26th of July Corridor, Zamalek, Cairo</t>
+          <t>Blue Lotus Wellbeing</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Facebook Events</t>
+          <t>AllEvents</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Campus &amp; Student Activities</t>
+          <t>General Event</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -7437,17 +7457,17 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Free Admission / Open to All Youth</t>
+          <t>Registration / Tickets</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>7.8</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -7457,27 +7477,27 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>campus, students, youth, education</t>
+          <t>general</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>Campus Outreach: Engage Student Attendees &amp; Student Union Partners</t>
+          <t>General Monitoring for potential youth presence</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>Make Friends Cairo Youth Community (@cairomakefriends)</t>
+          <t>AllEvents Organizer</t>
         </is>
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/cairomakefriends</t>
+          <t>https://allevents.in/heliopolis/chromatic-healing-level-2/200030583735256</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/groups/cairomakefriends</t>
+          <t>https://allevents.in/heliopolis/chromatic-healing-level-2/200030583735256</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
@@ -7485,11 +7505,7 @@
           <t>100% Verified Real</t>
         </is>
       </c>
-      <c r="R78" t="inlineStr">
-        <is>
-          <t>The most active youth and international student cultural exchange gathering in Greater Cairo. Convenes university students, foreign exchange delegates, language learners, and young professionals for cross-cultural dialogues and networking in Zamalek.</t>
-        </is>
-      </c>
+      <c r="R78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -7582,12 +7598,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>The Egypt Coffee Festival 2026</t>
+          <t>Mawlana Band at Room Garden city</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Oct 16, 17</t>
+          <t>Fri, 16 Oct, 2026 - 08:00 PM</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -7597,12 +7613,12 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Kamelizer Spaces, District 5</t>
+          <t>ROOM Art Space &amp; Cafe</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>TicketsMarche</t>
+          <t>AllEvents</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -7617,7 +7633,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>350.00 EGP</t>
+          <t>Registration / Tickets</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -7647,17 +7663,17 @@
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>Kamelizer sspaces</t>
+          <t>AllEvents Organizer</t>
         </is>
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>https://www.ticketsmarche.com/event/The_Egypt_Coffee_Festival_2026_9398</t>
+          <t>https://allevents.in/cairo/mawlana-band-at-room-garden-city/200030769947005</t>
         </is>
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>https://www.ticketsmarche.com/event/The_Egypt_Coffee_Festival_2026_9398</t>
+          <t>https://allevents.in/cairo/mawlana-band-at-room-garden-city/200030769947005</t>
         </is>
       </c>
       <c r="Q80" t="inlineStr">
@@ -7665,21 +7681,17 @@
           <t>100% Verified Real</t>
         </is>
       </c>
-      <c r="R80" t="inlineStr">
-        <is>
-          <t>The Egypt Coffee Festival 2026 organized by Kamelizer sspaces. Tickets available on TicketsMarche (350.00 EGP). Venue: Kamelizer Spaces, District 5.</t>
-        </is>
-      </c>
+      <c r="R80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Tul8te Live at Manara Arena</t>
+          <t>The Egypt Coffee Festival 2026</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Oct 16 · 05:00 PM</t>
+          <t>Oct 16, 17</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -7689,7 +7701,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Al Manara Arena</t>
+          <t>Kamelizer Spaces, District 5</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -7709,7 +7721,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1000.00 EGP</t>
+          <t>350.00 EGP</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -7739,17 +7751,17 @@
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>Urchin Experiences</t>
+          <t>Kamelizer sspaces</t>
         </is>
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>https://www.ticketsmarche.com/event/Tul8te_9353</t>
+          <t>https://www.ticketsmarche.com/event/The_Egypt_Coffee_Festival_2026_9398</t>
         </is>
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>https://www.ticketsmarche.com/event/Tul8te_9353</t>
+          <t>https://www.ticketsmarche.com/event/The_Egypt_Coffee_Festival_2026_9398</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr">
@@ -7759,19 +7771,19 @@
       </c>
       <c r="R81" t="inlineStr">
         <is>
-          <t>Tul8te Live at Manara Arena organized by Urchin Experiences. Tickets available on TicketsMarche (1000.00 EGP). Venue: Al Manara Arena.</t>
+          <t>The Egypt Coffee Festival 2026 organized by Kamelizer sspaces. Tickets available on TicketsMarche (350.00 EGP). Venue: Kamelizer Spaces, District 5.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Omar Khairat at Fustat Festival</t>
+          <t>Tul8te Live at Manara Arena</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Oct 16 · 10:00 PM</t>
+          <t>Oct 16 · 05:00 PM</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -7781,7 +7793,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Fustat</t>
+          <t>Al Manara Arena</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -7801,7 +7813,7 @@
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>1100.00 EGP</t>
+          <t>1000.00 EGP</t>
         </is>
       </c>
       <c r="I82" t="inlineStr">
@@ -7831,17 +7843,17 @@
       </c>
       <c r="N82" t="inlineStr">
         <is>
-          <t>Waleed Mansour</t>
+          <t>Urchin Experiences</t>
         </is>
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>https://www.ticketsmarche.com/event/omar_khairat_9481</t>
+          <t>https://www.ticketsmarche.com/event/Tul8te_9353</t>
         </is>
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>https://www.ticketsmarche.com/event/omar_khairat_9481</t>
+          <t>https://www.ticketsmarche.com/event/Tul8te_9353</t>
         </is>
       </c>
       <c r="Q82" t="inlineStr">
@@ -7851,19 +7863,19 @@
       </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t>Omar Khairat at Fustat Festival organized by Waleed Mansour. Tickets available on TicketsMarche (1100.00 EGP). Venue: Fustat.</t>
+          <t>Tul8te Live at Manara Arena organized by Urchin Experiences. Tickets available on TicketsMarche (1000.00 EGP). Venue: Al Manara Arena.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Mawlana Band at Room Garden city</t>
+          <t>Omar Khairat at Fustat Festival</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Fri, 16 Oct, 2026 - 08:00 PM</t>
+          <t>Oct 16 · 10:00 PM</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -7873,12 +7885,12 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>ROOM Art Space &amp; Cafe</t>
+          <t>Fustat</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>AllEvents</t>
+          <t>TicketsMarche</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -7893,7 +7905,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Registration / Tickets</t>
+          <t>1100.00 EGP</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -7923,17 +7935,17 @@
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>AllEvents Organizer</t>
+          <t>Waleed Mansour</t>
         </is>
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>https://allevents.in/cairo/mawlana-band-at-room-garden-city/200030769947005</t>
+          <t>https://www.ticketsmarche.com/event/omar_khairat_9481</t>
         </is>
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>https://allevents.in/cairo/mawlana-band-at-room-garden-city/200030769947005</t>
+          <t>https://www.ticketsmarche.com/event/omar_khairat_9481</t>
         </is>
       </c>
       <c r="Q83" t="inlineStr">
@@ -7941,7 +7953,11 @@
           <t>100% Verified Real</t>
         </is>
       </c>
-      <c r="R83" t="inlineStr"/>
+      <c r="R83" t="inlineStr">
+        <is>
+          <t>Omar Khairat at Fustat Festival organized by Waleed Mansour. Tickets available on TicketsMarche (1100.00 EGP). Venue: Fustat.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -8038,17 +8054,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>PACES LIVE- Communications &amp; Consultation Course</t>
+          <t>PACES LIVE- Communications &amp; Consultation  Course</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Sat, 17 Oct • 09:00 AM</t>
+          <t>Sat, 17 Oct, 2026 - 09:00 AM</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Tanta</t>
+          <t>Cairo</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -8126,17 +8142,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>BIODIESEL PRODUCTION TRAINING EGYPT 2026</t>
+          <t>Biodiesel Production Training Program 2026 Rounds</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Sat, 17 Oct • 09:00 AM</t>
+          <t>Sat, 17 Oct, 2026 - 09:00 AM</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Tanta</t>
+          <t>Cairo</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -8196,12 +8212,12 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>https://allevents.in/cairo/biodiesel-production-training-egypt-2026/200030723108408</t>
+          <t>https://allevents.in/cairo/biodiesel-production-training-program-2026-rounds/200030798987446</t>
         </is>
       </c>
       <c r="P86" t="inlineStr">
         <is>
-          <t>https://allevents.in/cairo/biodiesel-production-training-egypt-2026/200030723108408</t>
+          <t>https://allevents.in/cairo/biodiesel-production-training-program-2026-rounds/200030798987446</t>
         </is>
       </c>
       <c r="Q86" t="inlineStr">
@@ -8214,12 +8230,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Biodiesel Production Training Program 2026 Rounds</t>
+          <t>BIODIESEL PRODUCTION TRAINING  EGYPT 2026</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Sat, 17 Oct, 2026 - 09:00 AM</t>
+          <t>Sat, 17 Oct • 09:00 AM</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -8284,12 +8300,12 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>https://allevents.in/cairo/biodiesel-production-training-program-2026-rounds/200030798987446</t>
+          <t>https://allevents.in/cairo/biodiesel-production-training-egypt-2026/200030723108408</t>
         </is>
       </c>
       <c r="P87" t="inlineStr">
         <is>
-          <t>https://allevents.in/cairo/biodiesel-production-training-program-2026-rounds/200030798987446</t>
+          <t>https://allevents.in/cairo/biodiesel-production-training-egypt-2026/200030723108408</t>
         </is>
       </c>
       <c r="Q87" t="inlineStr">
@@ -8547,7 +8563,7 @@
       </c>
       <c r="N90" t="inlineStr">
         <is>
-          <t>AHC Advertising Agency</t>
+          <t>AHC Advertising  Agency</t>
         </is>
       </c>
       <c r="O90" t="inlineStr">
@@ -8567,7 +8583,7 @@
       </c>
       <c r="R90" t="inlineStr">
         <is>
-          <t>STEPS SUMMIT organized by AHC Advertising Agency. Tickets available on TicketsMarche (1000.00 EGP). Venue: SODIC Sports Club at SODIC East.</t>
+          <t>STEPS SUMMIT organized by AHC Advertising  Agency. Tickets available on TicketsMarche (1000.00 EGP). Venue: SODIC Sports Club at SODIC East.</t>
         </is>
       </c>
     </row>
@@ -8850,7 +8866,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>10 Days Sun Festival Egypt Tour Package Cairo Abu Simbel &amp; 3 Nights Nile Cruise</t>
+          <t>10 Days Sun Festival Egypt Tour Package  Cairo Abu Simbel &amp; 3 Nights Nile Cruise</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -9311,12 +9327,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Tue, 20 Oct • 10:00 AM</t>
+          <t>Tue, 20 Oct, 2026 - 10:00 AM</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Tanta</t>
+          <t>Cairo</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -9394,52 +9410,52 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Cairo Toastmasters Meeting - Develop your public speaking in Tagamo3!</t>
+          <t>BUE Youth Executive Leadership &amp; Entrepreneurship Forum</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Oct 20, 2026 · 04:00 PM</t>
+          <t>Oct 20, 2026 · 01:00 PM</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>New Cairo</t>
+          <t>Cairo</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Espaces</t>
+          <t>BUE The British University in Egypt, El Shorouk City, Cairo</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Meetup</t>
+          <t>Facebook Events</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Student Orgs &amp; Campus Leadership</t>
+          <t>University Conferences &amp; Academic Forums</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>Toastmasters</t>
+          <t>Student Union</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>Free</t>
+          <t>Registration Required / Certificate of Completion</t>
         </is>
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>8.7</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -9449,27 +9465,27 @@
       </c>
       <c r="L100" t="inlineStr">
         <is>
-          <t>Toastmasters, student, campus, youth, leadership</t>
+          <t>university, academic, conference, campus, youth</t>
         </is>
       </c>
       <c r="M100" t="inlineStr">
         <is>
-          <t>Partner Outreach with Toastmasters: Joint Activation / PR Collaboration</t>
+          <t>Major Campus Activation: Deploy Chapter Delegation, Booth Presence &amp; Recruit University Students</t>
         </is>
       </c>
       <c r="N100" t="inlineStr">
         <is>
-          <t>Cairo Toastmasters - Improve your Public Speaking!</t>
+          <t>The British University in Egypt (BUE) Student Union &amp; Business Faculty</t>
         </is>
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/cairotmclub/events/316705095/</t>
+          <t>https://www.bue.edu.eg/</t>
         </is>
       </c>
       <c r="P100" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/cairotmclub/events/316705095/</t>
+          <t>https://www.facebook.com/thebritishuniversityinegypt</t>
         </is>
       </c>
       <c r="Q100" t="inlineStr">
@@ -9479,59 +9495,59 @@
       </c>
       <c r="R100" t="inlineStr">
         <is>
-          <t>Do you want to kick your public speaking skills up a couple of notches? Join Cairo Toastmasters and practice public speaking with professional speakers from all over the world to ace your next presentation. Please join our whatsapp group to receive the invitation and meeting details. https://chat</t>
+          <t>Interactive youth executive leadership and entrepreneurship forum hosted at BUE campus in El Shorouk. Designed for business, law, engineering, and economics undergraduates seeking executive decision-making frameworks, startup incubation, and international career readiness.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>BUE Youth Executive Leadership &amp; Entrepreneurship Forum</t>
+          <t>Cairo Toastmasters Meeting - Develop your public speaking in Tagamo3!</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Oct 20, 2026 · 01:00 PM</t>
+          <t>Oct 20, 2026 · 04:00 PM</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Cairo</t>
+          <t>New Cairo</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>BUE The British University in Egypt, El Shorouk City, Cairo</t>
+          <t>Espaces</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Facebook Events</t>
+          <t>Meetup</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>University Conferences &amp; Academic Forums</t>
+          <t>Student Orgs &amp; Campus Leadership</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>Student Union</t>
+          <t>Toastmasters</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>Registration Required / Certificate of Completion</t>
+          <t>Free</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>8.7</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>HIGH</t>
+          <t>MEDIUM</t>
         </is>
       </c>
       <c r="K101" t="inlineStr">
@@ -9541,27 +9557,27 @@
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>university, academic, conference, campus, youth</t>
+          <t>Toastmasters, student, campus, youth, leadership</t>
         </is>
       </c>
       <c r="M101" t="inlineStr">
         <is>
-          <t>Major Campus Activation: Deploy Chapter Delegation, Booth Presence &amp; Recruit University Students</t>
+          <t>Partner Outreach with Toastmasters: Joint Activation / PR Collaboration</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t>The British University in Egypt (BUE) Student Union &amp; Business Faculty</t>
+          <t>Cairo Toastmasters - Improve your Public Speaking!</t>
         </is>
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>https://www.bue.edu.eg/</t>
+          <t>https://www.meetup.com/cairotmclub/events/316705095/</t>
         </is>
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/thebritishuniversityinegypt</t>
+          <t>https://www.meetup.com/cairotmclub/events/316705095/</t>
         </is>
       </c>
       <c r="Q101" t="inlineStr">
@@ -9571,7 +9587,10 @@
       </c>
       <c r="R101" t="inlineStr">
         <is>
-          <t>Interactive youth executive leadership and entrepreneurship forum hosted at BUE campus in El Shorouk. Designed for business, law, engineering, and economics undergraduates seeking executive decision-making frameworks, startup incubation, and international career readiness.</t>
+          <t>Do you want to kick your public speaking skills up a couple of notches?
+Join Cairo Toastmasters and practice public speaking with professional speakers from all over the world to ace your next presentation.
+Please join our whatsapp group to receive the invitation and meeting details.
+https://chat</t>
         </is>
       </c>
     </row>
@@ -9935,7 +9954,10 @@
       </c>
       <c r="R105" t="inlineStr">
         <is>
-          <t>Do you want to kick your public speaking skills up a couple of notches? Join Inspire Toastmasters Club and practice public speaking with professional speakers from all over the world to ace your next presentation. What's Inspire Toastmasters Club? A Toastmasters Club meeting is a learn-by-doing e</t>
+          <t>Do you want to kick your public speaking skills up a couple of notches?
+Join Inspire Toastmasters Club and practice public speaking with professional speakers from all over the world to ace your next presentation.
+What's Inspire Toastmasters Club?
+A Toastmasters Club meeting is a learn-by-doing e</t>
         </is>
       </c>
     </row>
@@ -10030,7 +10052,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>3x1 _ _</t>
+          <t>3x1  _ _</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -11116,7 +11138,7 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Tanta</t>
+          <t>Cairo</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -11929,7 +11951,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Cineolios Cinenights Alexandria</t>
+          <t>Cineolios Cinenights  Alexandria</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -13470,12 +13492,12 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Thu, 29 Oct • 10:00 AM</t>
+          <t>Thu, 29 Oct, 2026 - 10:00 AM</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Tanta</t>
+          <t>Cairo</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
@@ -14651,17 +14673,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>17th Arab Diabetes Forum ADF 2026.</t>
+          <t>17th Arab Diabetes Forum  ADF 2026.</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Tue, 03 Nov • 08:00 AM</t>
+          <t>Tue, 03 Nov, 2026 - 08:00 AM</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Tanta</t>
+          <t>Cairo</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -14919,12 +14941,12 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Inspire Toastmasters Club Meeting</t>
+          <t>برنامج التدريب الطبي الطلابي الخامس - 'الومضة الخامسة' 2026</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Nov 04, 2026 · 05:00 PM</t>
+          <t>Nov 04, 2026 · 10:00 AM</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -14934,32 +14956,32 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>MQR, The Greek Compus</t>
+          <t>Club De La Salle, Daher, Cairo</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>Meetup</t>
+          <t>Facebook Events</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>Student Orgs &amp; Campus Leadership</t>
+          <t>Youth Leadership &amp; Skills Workshops</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>Toastmasters</t>
+          <t>Independent</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>Free</t>
+          <t>Free Student Enrollment</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>8.0</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
@@ -14974,27 +14996,27 @@
       </c>
       <c r="L161" t="inlineStr">
         <is>
-          <t>Toastmasters, student, campus, youth, leadership</t>
+          <t>workshop, skills, leadership, development</t>
         </is>
       </c>
       <c r="M161" t="inlineStr">
         <is>
-          <t>Partner Outreach with Toastmasters: Joint Activation / PR Collaboration</t>
+          <t>Speaker Outreach, Workshop Co-hosting &amp; Youth Leadership Presentation</t>
         </is>
       </c>
       <c r="N161" t="inlineStr">
         <is>
-          <t>Cairo Toastmasters - Improve your Public Speaking!</t>
+          <t>Club De La Salle Medical Student Committee &amp; IFMSA Egypt</t>
         </is>
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/cairotmclub/events/316296322/</t>
+          <t>https://ifmsa.eg/</t>
         </is>
       </c>
       <c r="P161" t="inlineStr">
         <is>
-          <t>https://www.meetup.com/cairotmclub/events/316296322/</t>
+          <t>https://ifmsa.eg/</t>
         </is>
       </c>
       <c r="Q161" t="inlineStr">
@@ -15004,19 +15026,19 @@
       </c>
       <c r="R161" t="inlineStr">
         <is>
-          <t>Do you want to kick your public speaking skills up a couple of notches? Join Inspire Toastmasters Club and practice public speaking with professional speakers from all over the world to ace your next presentation. What's Inspire Toastmasters Club? A Toastmasters Club meeting is a learn-by-doing e</t>
+          <t>برنامج تدريبي متقدم يستهدف طلاب كليات الطب والصيدلة والتمريض بمختلف الجامعات المصرية. يركز على مهارات التواصل مع المرضى، الإسعافات الأولية المتقدمة، وإدارة الفرق الطبية التطوعية في القوافل العلاجية.</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>برنامج التدريب الطبي الطلابي الخامس - 'الومضة الخامسة' 2026</t>
+          <t>Inspire Toastmasters Club Meeting</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Nov 04, 2026 · 10:00 AM</t>
+          <t>Nov 04, 2026 · 05:00 PM</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -15026,32 +15048,32 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Club De La Salle, Daher, Cairo</t>
+          <t>MQR, The Greek Compus</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Facebook Events</t>
+          <t>Meetup</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>Youth Leadership &amp; Skills Workshops</t>
+          <t>Student Orgs &amp; Campus Leadership</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>Independent</t>
+          <t>Toastmasters</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>Free Student Enrollment</t>
+          <t>Free</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>8.0</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
@@ -15066,27 +15088,27 @@
       </c>
       <c r="L162" t="inlineStr">
         <is>
-          <t>workshop, skills, leadership, development</t>
+          <t>Toastmasters, student, campus, youth, leadership</t>
         </is>
       </c>
       <c r="M162" t="inlineStr">
         <is>
-          <t>Speaker Outreach, Workshop Co-hosting &amp; Youth Leadership Presentation</t>
+          <t>Partner Outreach with Toastmasters: Joint Activation / PR Collaboration</t>
         </is>
       </c>
       <c r="N162" t="inlineStr">
         <is>
-          <t>Club De La Salle Medical Student Committee &amp; IFMSA Egypt</t>
+          <t>Cairo Toastmasters - Improve your Public Speaking!</t>
         </is>
       </c>
       <c r="O162" t="inlineStr">
         <is>
-          <t>https://ifmsa.eg/</t>
+          <t>https://www.meetup.com/cairotmclub/events/316296322/</t>
         </is>
       </c>
       <c r="P162" t="inlineStr">
         <is>
-          <t>https://ifmsa.eg/</t>
+          <t>https://www.meetup.com/cairotmclub/events/316296322/</t>
         </is>
       </c>
       <c r="Q162" t="inlineStr">
@@ -15096,7 +15118,10 @@
       </c>
       <c r="R162" t="inlineStr">
         <is>
-          <t>برنامج تدريبي متقدم يستهدف طلاب كليات الطب والصيدلة والتمريض بمختلف الجامعات المصرية. يركز على مهارات التواصل مع المرضى، الإسعافات الأولية المتقدمة، وإدارة الفرق الطبية التطوعية في القوافل العلاجية.</t>
+          <t>Do you want to kick your public speaking skills up a couple of notches?
+Join Inspire Toastmasters Club and practice public speaking with professional speakers from all over the world to ace your next presentation.
+What's Inspire Toastmasters Club?
+A Toastmasters Club meeting is a learn-by-doing e</t>
         </is>
       </c>
     </row>
@@ -16096,12 +16121,12 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Fri, 06 Nov • 09:00 AM</t>
+          <t>Fri, 06 Nov, 2026 - 09:00 AM</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Tanta</t>
+          <t>Cairo</t>
         </is>
       </c>
       <c r="D174" t="inlineStr">
@@ -17542,7 +17567,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2nd MYTHS FACTS in Pediatric Practice</t>
+          <t>2nd MYTHS  FACTS in Pediatric Practice</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -17630,22 +17655,22 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Mansoura Chest Department Annual Conference 2026</t>
+          <t>FEGO Egypt Womens Health Congress 2026</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Thu, 12 Nov • 08:00 AM</t>
+          <t>Thu, 12 Nov, 2026 - 08:00 AM</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Mansoura</t>
+          <t>Cairo</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Port Fouad</t>
+          <t>Le Méridien Cairo Airport</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
@@ -17700,12 +17725,12 @@
       </c>
       <c r="O191" t="inlineStr">
         <is>
-          <t>https://allevents.in/port-said/mansoura-chest-department-annual-conference-2026/200030669991447</t>
+          <t>https://allevents.in/cairo/fego-egypt-womens-health-congress-2026/200030803418648</t>
         </is>
       </c>
       <c r="P191" t="inlineStr">
         <is>
-          <t>https://allevents.in/port-said/mansoura-chest-department-annual-conference-2026/200030669991447</t>
+          <t>https://allevents.in/cairo/fego-egypt-womens-health-congress-2026/200030803418648</t>
         </is>
       </c>
       <c r="Q191" t="inlineStr">
@@ -17718,22 +17743,22 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>FEGO Egypt Womens Health Congress 2026</t>
+          <t>Mansoura Chest Department Annual Conference 2026</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Thu, 12 Nov, 2026 - 08:00 AM</t>
+          <t>Thu, 12 Nov • 08:00 AM</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Cairo</t>
+          <t>Mansoura</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Le Méridien Cairo Airport</t>
+          <t>Port Fouad</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
@@ -17788,12 +17813,12 @@
       </c>
       <c r="O192" t="inlineStr">
         <is>
-          <t>https://allevents.in/cairo/fego-egypt-womens-health-congress-2026/200030803418648</t>
+          <t>https://allevents.in/port-said/mansoura-chest-department-annual-conference-2026/200030669991447</t>
         </is>
       </c>
       <c r="P192" t="inlineStr">
         <is>
-          <t>https://allevents.in/cairo/fego-egypt-womens-health-congress-2026/200030803418648</t>
+          <t>https://allevents.in/port-said/mansoura-chest-department-annual-conference-2026/200030669991447</t>
         </is>
       </c>
       <c r="Q192" t="inlineStr">
@@ -18166,12 +18191,12 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Max Amini Live in Cairo</t>
+          <t>Masters behind the microscope</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Nov 12,13 &amp; 14</t>
+          <t>Thu, 12 Nov, 2026 - 11:00 PM</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -18181,12 +18206,12 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>St. Regis, New Capital</t>
+          <t>Hilton Grand Nile -Cairo</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>TicketsMarche, AllEvents</t>
+          <t>AllEvents</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
@@ -18201,7 +18226,7 @@
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>Free / Paid Tickets</t>
+          <t>Registration / Tickets</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
@@ -18231,17 +18256,17 @@
       </c>
       <c r="N197" t="inlineStr">
         <is>
-          <t>ACUD\u0026LN</t>
+          <t>AllEvents Organizer</t>
         </is>
       </c>
       <c r="O197" t="inlineStr">
         <is>
-          <t>https://www.ticketsmarche.com/event/MaxAmini-9128</t>
+          <t>https://allevents.in/cairo/masters-behind-the-microscope/200030565007741</t>
         </is>
       </c>
       <c r="P197" t="inlineStr">
         <is>
-          <t>https://www.ticketsmarche.com/event/MaxAmini-9128</t>
+          <t>https://allevents.in/cairo/masters-behind-the-microscope/200030565007741</t>
         </is>
       </c>
       <c r="Q197" t="inlineStr">
@@ -18249,31 +18274,27 @@
           <t>100% Verified Real</t>
         </is>
       </c>
-      <c r="R197" t="inlineStr">
-        <is>
-          <t>Max Amini Live in Cairo organized by ACUD\u0026LN. Tickets available on TicketsMarche (Free / Paid Tickets). Venue: St. Regis, New Capital.</t>
-        </is>
-      </c>
+      <c r="R197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Masters behind the microscope</t>
+          <t>(SHEDA) Celebrating World Diabetes Day " Early Action on Diabetes "</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Thu, 12 Nov, 2026 - 11:00 PM</t>
+          <t>Fri, 13 Nov • 08:00 AM</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>Cairo</t>
+          <t>Mansoura</t>
         </is>
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Hilton Grand Nile -Cairo</t>
+          <t>Grand Hotel Port Said -  جراند اوتيل بورسعيد</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
@@ -18328,12 +18349,12 @@
       </c>
       <c r="O198" t="inlineStr">
         <is>
-          <t>https://allevents.in/cairo/masters-behind-the-microscope/200030565007741</t>
+          <t>https://allevents.in/port-said/sheda-celebrating-world-diabetes-day-early-action-on-diabetes/200030407263926</t>
         </is>
       </c>
       <c r="P198" t="inlineStr">
         <is>
-          <t>https://allevents.in/cairo/masters-behind-the-microscope/200030565007741</t>
+          <t>https://allevents.in/port-said/sheda-celebrating-world-diabetes-day-early-action-on-diabetes/200030407263926</t>
         </is>
       </c>
       <c r="Q198" t="inlineStr">
@@ -18346,22 +18367,22 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>(SHEDA) Celebrating World Diabetes Day " Early Action on Diabetes "</t>
+          <t>5th Annual Conference of the Dermatology Department  Zagazig General Hospital</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Fri, 13 Nov • 08:00 AM</t>
+          <t>Fri, 13 Nov, 2026 - 08:00 AM</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Mansoura</t>
+          <t>Sharkia</t>
         </is>
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Grand Hotel Port Said -  جراند اوتيل بورسعيد</t>
+          <t>Triumph Luxury Hotel</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
@@ -18371,7 +18392,7 @@
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>General Event</t>
+          <t>Medical &amp; Clinical Congress</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
@@ -18386,7 +18407,7 @@
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>2.5</t>
         </is>
       </c>
       <c r="J199" t="inlineStr">
@@ -18396,17 +18417,17 @@
       </c>
       <c r="K199" t="inlineStr">
         <is>
-          <t>⚠️ Clash</t>
+          <t>Clear</t>
         </is>
       </c>
       <c r="L199" t="inlineStr">
         <is>
-          <t>general</t>
+          <t>medical, clinical, b2b</t>
         </is>
       </c>
       <c r="M199" t="inlineStr">
         <is>
-          <t>General Monitoring for potential youth presence</t>
+          <t>Do Not Deploy (Niche Clinical Target - Incompatible with Youth B2C)</t>
         </is>
       </c>
       <c r="N199" t="inlineStr">
@@ -18416,12 +18437,12 @@
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>https://allevents.in/port-said/sheda-celebrating-world-diabetes-day-early-action-on-diabetes/200030407263926</t>
+          <t>https://allevents.in/cairo/5th-annual-conference-of-the-dermatology-department-zagazig-general-hospital/200030600400453</t>
         </is>
       </c>
       <c r="P199" t="inlineStr">
         <is>
-          <t>https://allevents.in/port-said/sheda-celebrating-world-diabetes-day-early-action-on-diabetes/200030407263926</t>
+          <t>https://allevents.in/cairo/5th-annual-conference-of-the-dermatology-department-zagazig-general-hospital/200030600400453</t>
         </is>
       </c>
       <c r="Q199" t="inlineStr">
@@ -18434,32 +18455,32 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>5th Annual Conference of the Dermatology Department Zagazig General Hospital</t>
+          <t>Max Amini Live in Cairo</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Fri, 13 Nov, 2026 - 08:00 AM</t>
+          <t>Fri, 13 Nov, 2026 - 05:00 PM</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Sharkia</t>
+          <t>Cairo</t>
         </is>
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Triumph Luxury Hotel</t>
+          <t>The St. Regis New Capital Cairo</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>AllEvents</t>
+          <t>AllEvents, TicketsMarche</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>Medical &amp; Clinical Congress</t>
+          <t>General Event</t>
         </is>
       </c>
       <c r="G200" t="inlineStr">
@@ -18474,7 +18495,7 @@
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>2.5</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="J200" t="inlineStr">
@@ -18484,17 +18505,17 @@
       </c>
       <c r="K200" t="inlineStr">
         <is>
-          <t>Clear</t>
+          <t>⚠️ Clash</t>
         </is>
       </c>
       <c r="L200" t="inlineStr">
         <is>
-          <t>medical, clinical, b2b</t>
+          <t>general</t>
         </is>
       </c>
       <c r="M200" t="inlineStr">
         <is>
-          <t>Do Not Deploy (Niche Clinical Target - Incompatible with Youth B2C)</t>
+          <t>General Monitoring for potential youth presence</t>
         </is>
       </c>
       <c r="N200" t="inlineStr">
@@ -18504,12 +18525,12 @@
       </c>
       <c r="O200" t="inlineStr">
         <is>
-          <t>https://allevents.in/cairo/5th-annual-conference-of-the-dermatology-department-zagazig-general-hospital/200030600400453</t>
+          <t>https://allevents.in/cairo/max-amini-live-in-cairo/200030638545421</t>
         </is>
       </c>
       <c r="P200" t="inlineStr">
         <is>
-          <t>https://allevents.in/cairo/5th-annual-conference-of-the-dermatology-department-zagazig-general-hospital/200030600400453</t>
+          <t>https://allevents.in/cairo/max-amini-live-in-cairo/200030638545421</t>
         </is>
       </c>
       <c r="Q200" t="inlineStr">
@@ -18517,7 +18538,11 @@
           <t>100% Verified Real</t>
         </is>
       </c>
-      <c r="R200" t="inlineStr"/>
+      <c r="R200" t="inlineStr">
+        <is>
+          <t>Max Amini Live in Cairo organized by ACUD\u0026LN. Tickets available on TicketsMarche (Free / Paid Tickets). Venue: St. Regis, New Capital.</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -19341,7 +19366,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>EGYVASC2026 19th -22th November 2026 Makadi bay Hurghada</t>
+          <t>EGYVASC2026 19th -22th November 2026 Makadi bay  Hurghada</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -20049,7 +20074,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>Assiut University Youth &amp; Technology Conclave</t>
+          <t>مؤتمر Paradox للقيادات الشبابية وريادة الأعمال بصعيد مصر</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -20069,7 +20094,7 @@
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>Egypt Flagship Summits</t>
+          <t>Egypt Flagship Summits, Facebook Events</t>
         </is>
       </c>
       <c r="F218" t="inlineStr">
@@ -20089,7 +20114,7 @@
       </c>
       <c r="I218" t="inlineStr">
         <is>
-          <t>9.8</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="J218" t="inlineStr">
@@ -20104,7 +20129,7 @@
       </c>
       <c r="L218" t="inlineStr">
         <is>
-          <t>IEEE, summit, flagship, youth, leadership</t>
+          <t>IEEE, student, campus, youth, leadership</t>
         </is>
       </c>
       <c r="M218" t="inlineStr">
@@ -21025,7 +21050,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>e-AGE26: المؤتمر السنوي السادس عشر - الأهرامات: بنيان لا يزول</t>
+          <t>e-AGE26</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -21045,7 +21070,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>AllEvents, Facebook Events</t>
+          <t>AllEvents</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
@@ -21065,12 +21090,12 @@
       </c>
       <c r="I229" t="inlineStr">
         <is>
-          <t>7.8</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="J229" t="inlineStr">
         <is>
-          <t>MEDIUM</t>
+          <t>LOW</t>
         </is>
       </c>
       <c r="K229" t="inlineStr">
@@ -21080,7 +21105,7 @@
       </c>
       <c r="L229" t="inlineStr">
         <is>
-          <t>general, campus, students, youth, education</t>
+          <t>general</t>
         </is>
       </c>
       <c r="M229" t="inlineStr">
@@ -21100,7 +21125,7 @@
       </c>
       <c r="P229" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/events/1880065419619587/</t>
+          <t>https://allevents.in/alexandria/e-age26-المؤتمر-السنوي-السادس-عشر-الأهرامات-بنيان-لا-يزول/200030323061248</t>
         </is>
       </c>
       <c r="Q229" t="inlineStr">
@@ -21108,14 +21133,7 @@
           <t>100% Verified Real</t>
         </is>
       </c>
-      <c r="R229" t="inlineStr">
-        <is>
-          <t>Tue, Dec 1 - Dec 3
-e-AGE26: المؤتمر السنوي السادس عشر - الأهرامات: بنيان لا يزول
-Chatby, Alexandria 21526, EGYPT, Alexandria, Egypt, P.O. Box 138
-3.1K interested · 115 going</t>
-        </is>
-      </c>
+      <c r="R229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -21564,7 +21582,7 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>El Gouna Photo Week</t>
+          <t>El Gouna Photo Week 2026</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
@@ -21584,7 +21602,7 @@
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>TicketsMarche</t>
+          <t>TicketsMarche, AllEvents</t>
         </is>
       </c>
       <c r="F235" t="inlineStr">
@@ -23982,7 +24000,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>EDUGATE Cairo 20th Edition – International Universities Fair</t>
+          <t>EDUGATE Cairo 20th Edition  International Universities Fair</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -24002,7 +24020,7 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>AllEvents, Eventbrite</t>
+          <t>AllEvents</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
@@ -24065,11 +24083,7 @@
           <t>100% Verified Real</t>
         </is>
       </c>
-      <c r="R262" t="inlineStr">
-        <is>
-          <t>EDUGATE Cairo 20th Edition is an international universities fair taking place from 1–3 February 2027 at Royal Maxim Palace Kempinski, Cairo.</t>
-        </is>
-      </c>
+      <c r="R262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">

</xml_diff>